<commit_message>
Polish portfolio oversight with public walkthrough and verified reporting
</commit_message>
<xml_diff>
--- a/outputs/oversight/Portfolio_Oversight.xlsx
+++ b/outputs/oversight/Portfolio_Oversight.xlsx
@@ -23,7 +23,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Decision'!$A$4:$C$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Decision'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Controls'!$A$4:$F$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Controls'!$A$4:$I$119</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Controls'!$1:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Exceptions'!$A$4:$J$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Exceptions'!$1:$4</definedName>
@@ -35,13 +35,13 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'Stress'!$1:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Reconciliation'!$A$4:$B$16</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'Reconciliation'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'PathMetrics'!$A$4:$H$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'PathMetrics'!$A$4:$N$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'PathMetrics'!$1:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'LinkedTotals'!$A$4:$G$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'LinkedTotals'!$1:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Contributions'!$A$4:$F$244</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="9">'Contributions'!$1:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'RunEvidence'!$A$4:$B$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'RunEvidence'!$A$4:$B$21</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="10">'RunEvidence'!$1:$4</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -654,7 +654,7 @@
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>oversight-20261012T234925</t>
+          <t>oversight-20261013T034644</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -7012,7 +7012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -7055,7 +7055,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>oversight-20261012T234925</t>
+          <t>oversight-20261013T034644</t>
         </is>
       </c>
     </row>
@@ -7067,7 +7067,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>2026-10-12T23:49:25.170427+00:00</t>
+          <t>2026-10-13T03:46:44.875025+00:00</t>
         </is>
       </c>
     </row>
@@ -7079,7 +7079,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-12T23:51:32.067685+00:00</t>
+          <t>2026-10-13T03:48:42.488421+00:00</t>
         </is>
       </c>
     </row>
@@ -7090,7 +7090,7 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>126.897</v>
+        <v>117.61</v>
       </c>
     </row>
     <row r="9">
@@ -7167,7 +7167,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>{"data/wrds/calendar.csv": "69b684681dd34a2fdc662563a3e060cb7d86b71e4f7d8cea9f8f6ac95938b53a", "data/wrds/daily.csv": "696aa0f881c6c95bb9cbd6536d82d71e0589221bae18f04932602a492bea0711", "data/wrds/identities.csv": "77b06ec307a732a2c62840da34279709f5c9ca0985f18636e01a06c1a08befcb", "data/wrds/manifest.json": "858e366756894b53a60dcb68c3b00178cc8476ae6fbdcee98cce698c8f0227f9", "outputs/wrds/run_summary.json": "54d81352ddc366b6fd76cfc7e55f361a79820526b5172d16e6390b1c7d4e05b3", "outputs/wrds_private/benchmark.csv": "3187c3a72d373e4836990ceb0c17bc0de81526fddddade09b290f2ec9fa6e323", "outputs/wrds_private/daily.csv": "3daf7e074a460de197f3d81a4e25d75b768d7167c56af4496ba77d90960abc0d", "outputs/wrds_private/decisions.csv": "1f74a5fcbe9475d5bf9a24555a3da346deb1f6b1d6ba586d21cf3c07efa217a1", "outputs/wrds_private/trades.csv": "ee5dee0a384c899ddd52a43835ce1d77cb189ff1df33ee48350bce6d538c9f91"}</t>
+          <t>{"data/wrds/calendar.csv": "69b684681dd34a2fdc662563a3e060cb7d86b71e4f7d8cea9f8f6ac95938b53a", "data/wrds/daily.csv": "696aa0f881c6c95bb9cbd6536d82d71e0589221bae18f04932602a492bea0711", "data/wrds/identities.csv": "77b06ec307a732a2c62840da34279709f5c9ca0985f18636e01a06c1a08befcb", "data/wrds/manifest.json": "858e366756894b53a60dcb68c3b00178cc8476ae6fbdcee98cce698c8f0227f9", "outputs/wrds/run_summary.json": "54d81352ddc366b6fd76cfc7e55f361a79820526b5172d16e6390b1c7d4e05b3", "outputs/wrds/scenario_summary.csv": "55d48175d52c1b023da7feec82f46b670c07b39a97ddc6e82a6b5d6abdd2a805", "outputs/wrds_private/benchmark.csv": "3187c3a72d373e4836990ceb0c17bc0de81526fddddade09b290f2ec9fa6e323", "outputs/wrds_private/daily.csv": "3daf7e074a460de197f3d81a4e25d75b768d7167c56af4496ba77d90960abc0d", "outputs/wrds_private/decisions.csv": "1f74a5fcbe9475d5bf9a24555a3da346deb1f6b1d6ba586d21cf3c07efa217a1", "outputs/wrds_private/trades.csv": "ee5dee0a384c899ddd52a43835ce1d77cb189ff1df33ee48350bce6d538c9f91"}</t>
         </is>
       </c>
     </row>
@@ -7179,60 +7179,72 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>{"oversight_contract.json": "b1a15ed553d313012bf22ddfe952e7aceabeb04d75f37febd225c5aaf612bb1a", "oversight_core.py": "50ffbe09e36b8eb369227aa2ef27e4fef7335a6aa5cc2e43b75e3066271ab747", "run_oversight.py": "4a594962d3812fb1cf4f9299de917d0378e00b02b841151df6f955f81666b492", "sql/oversight_daily_controls.sql": "7503d3ffd72f652b9ea472afe816bb0e0abf0ce9de61fad196a5ca35b8cf4837", "sql/oversight_trade_controls.sql": "bd22992db2a27ebc9266f7c36fa674f6b82376a3823f39360fb5e0a1842be44f"}</t>
+          <t>{"oversight_contract.json": "b1a15ed553d313012bf22ddfe952e7aceabeb04d75f37febd225c5aaf612bb1a", "oversight_core.py": "1bae6943b0dc77e4085414a0e597d8781ae466f59f2fb2f9a7a9b3934e249236", "run_oversight.py": "c379a54fc7304c8c87b01bb26e944e31a291bb8eaef952d23628bca9bda2a8cf", "sql/oversight_daily_controls.sql": "7503d3ffd72f652b9ea472afe816bb0e0abf0ce9de61fad196a5ca35b8cf4837", "sql/oversight_trade_controls.sql": "bd22992db2a27ebc9266f7c36fa674f6b82376a3823f39360fb5e0a1842be44f"}</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>public_artifact_sha256</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>{"outputs/oversight/historical_stress.json": "43b70392b29d14943a0f64009fe25e2d6cd92af03acce29438e38693a831591f", "outputs/oversight/incident_summary.json": "cea6c97b496d7dec3b601bd88f9045e08018da164ac9e8699f45c6f9fb77f0e0", "outputs/oversight/validation_summary.json": "afba2f564c2ed687e8c7c9c5374ccbfe857e49812d194e24d55703df96fbd303", "outputs/wrds/scenario_summary.csv": "55d48175d52c1b023da7feec82f46b670c07b39a97ddc6e82a6b5d6abdd2a805"}</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>interpretation</t>
+          <t>status</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Technical evidence-release decision only. Not investment approval, an actual order gate, or a claim of future alpha.</t>
+          <t>PASS</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>source</t>
+          <t>interpretation</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Existing WRDS/CRSP current-vintage historical research; no fresh market-data retrieval.</t>
+          <t>Technical evidence-release decision only. Not investment approval, an actual order gate, or a claim of future alpha.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Existing WRDS/CRSP current-vintage historical research; no fresh market-data retrieval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
           <t>privacy</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B21" s="4" t="inlineStr">
         <is>
           <t>Only aggregate challenger/incident/stress receipts are public. Security-day source, detailed holdings, contributions and trades remain local.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:B20"/>
+  <autoFilter ref="A4:B21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -7499,7 +7511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F119"/>
+  <dimension ref="A1:I119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="47" customWidth="1" min="1" max="1"/>
@@ -7508,6 +7520,9 @@
     <col width="24" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="31" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -7521,11 +7536,14 @@
       <c r="D1" s="1" t="n"/>
       <c r="E1" s="1" t="n"/>
       <c r="F1" s="1" t="n"/>
+      <c r="G1" s="1" t="n"/>
+      <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>PASS is technical consistency. A passing control is not proof the investment decision is optimal.</t>
+          <t>Residual and tolerance share the explicit unit column. PASS is technical consistency, not investment approval.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -7533,6 +7551,9 @@
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -7565,6 +7586,21 @@
           <t>detail</t>
         </is>
       </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>category_label</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -7587,6 +7623,21 @@
         <v>0</v>
       </c>
       <c r="F5" s="4" t="inlineStr"/>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>governance</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Configuration and provenance</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -7600,7 +7651,7 @@
         </is>
       </c>
       <c r="C6" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>0</v>
@@ -7609,6 +7660,21 @@
         <v>0</v>
       </c>
       <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>governance</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Configuration and provenance</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -7622,7 +7688,7 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>0</v>
@@ -7635,6 +7701,21 @@
           <t>Detailed reconstructed holdings and returns may only be written under outputs/oversight_private.</t>
         </is>
       </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>governance</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Configuration and provenance</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -7661,6 +7742,21 @@
           <t>UTF-8 source fingerprint with CRLF/CR normalized to LF; substantive source changes still block.</t>
         </is>
       </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="inlineStr">
+        <is>
+          <t>governance</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>Configuration and provenance</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -7687,6 +7783,21 @@
           <t>UTF-8 source fingerprint with CRLF/CR normalized to LF; substantive source changes still block.</t>
         </is>
       </c>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>governance</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr">
+        <is>
+          <t>Configuration and provenance</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -7713,6 +7824,21 @@
           <t>UTF-8 source fingerprint with CRLF/CR normalized to LF; substantive source changes still block.</t>
         </is>
       </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H10" s="5" t="inlineStr">
+        <is>
+          <t>governance</t>
+        </is>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Configuration and provenance</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -7735,6 +7861,21 @@
         <v>0</v>
       </c>
       <c r="F11" s="4" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>governance</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>Configuration and provenance</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -7757,6 +7898,21 @@
         <v>0</v>
       </c>
       <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t>governance</t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>Configuration and provenance</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -7779,6 +7935,21 @@
         <v>0</v>
       </c>
       <c r="F13" s="4" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>governance</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Configuration and provenance</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -7801,6 +7972,21 @@
         <v>0</v>
       </c>
       <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>governance</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>Configuration and provenance</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -7823,6 +8009,21 @@
         <v>0</v>
       </c>
       <c r="F15" s="4" t="inlineStr"/>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>governance</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr">
+        <is>
+          <t>Configuration and provenance</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -7845,6 +8046,21 @@
         <v>0</v>
       </c>
       <c r="F16" s="5" t="inlineStr"/>
+      <c r="G16" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>governance</t>
+        </is>
+      </c>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>Configuration and provenance</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -7867,6 +8083,21 @@
         <v>0</v>
       </c>
       <c r="F17" s="4" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H17" s="4" t="inlineStr">
+        <is>
+          <t>governance</t>
+        </is>
+      </c>
+      <c r="I17" s="4" t="inlineStr">
+        <is>
+          <t>Configuration and provenance</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -7893,6 +8124,21 @@
           <t>Required columns present.</t>
         </is>
       </c>
+      <c r="G18" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -7915,6 +8161,21 @@
         <v>0</v>
       </c>
       <c r="F19" s="4" t="inlineStr"/>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -7937,6 +8198,21 @@
         <v>0</v>
       </c>
       <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -7959,6 +8235,21 @@
         <v>0</v>
       </c>
       <c r="F21" s="4" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -7981,6 +8272,21 @@
         <v>0</v>
       </c>
       <c r="F22" s="5" t="inlineStr"/>
+      <c r="G22" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I22" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -8003,6 +8309,21 @@
         <v>0</v>
       </c>
       <c r="F23" s="4" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -8029,6 +8350,21 @@
           <t>Required columns present.</t>
         </is>
       </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I24" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -8051,6 +8387,21 @@
         <v>0</v>
       </c>
       <c r="F25" s="4" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H25" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
@@ -8073,6 +8424,21 @@
         <v>0</v>
       </c>
       <c r="F26" s="5" t="inlineStr"/>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -8095,6 +8461,21 @@
         <v>0</v>
       </c>
       <c r="F27" s="4" t="inlineStr"/>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
@@ -8121,6 +8502,21 @@
           <t>Required columns present.</t>
         </is>
       </c>
+      <c r="G28" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -8143,6 +8539,21 @@
         <v>0</v>
       </c>
       <c r="F29" s="4" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -8165,6 +8576,21 @@
         <v>0</v>
       </c>
       <c r="F30" s="5" t="inlineStr"/>
+      <c r="G30" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I30" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -8187,6 +8613,21 @@
         <v>0</v>
       </c>
       <c r="F31" s="4" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -8209,6 +8650,21 @@
         <v>0</v>
       </c>
       <c r="F32" s="5" t="inlineStr"/>
+      <c r="G32" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I32" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -8231,6 +8687,21 @@
         <v>0</v>
       </c>
       <c r="F33" s="4" t="inlineStr"/>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -8257,6 +8728,21 @@
           <t>Required columns present.</t>
         </is>
       </c>
+      <c r="G34" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -8279,6 +8765,21 @@
         <v>0</v>
       </c>
       <c r="F35" s="4" t="inlineStr"/>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H35" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -8301,6 +8802,21 @@
         <v>0</v>
       </c>
       <c r="F36" s="5" t="inlineStr"/>
+      <c r="G36" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -8323,6 +8839,21 @@
         <v>0</v>
       </c>
       <c r="F37" s="4" t="inlineStr"/>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H37" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -8345,6 +8876,21 @@
         <v>0</v>
       </c>
       <c r="F38" s="5" t="inlineStr"/>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I38" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -8367,6 +8913,21 @@
         <v>0</v>
       </c>
       <c r="F39" s="4" t="inlineStr"/>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H39" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -8393,6 +8954,21 @@
           <t>Required columns present.</t>
         </is>
       </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -8415,6 +8991,21 @@
         <v>0</v>
       </c>
       <c r="F41" s="4" t="inlineStr"/>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H41" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
@@ -8437,6 +9028,21 @@
         <v>0</v>
       </c>
       <c r="F42" s="5" t="inlineStr"/>
+      <c r="G42" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -8459,6 +9065,21 @@
         <v>0</v>
       </c>
       <c r="F43" s="4" t="inlineStr"/>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
@@ -8481,6 +9102,21 @@
         <v>0</v>
       </c>
       <c r="F44" s="5" t="inlineStr"/>
+      <c r="G44" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I44" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -8503,6 +9139,21 @@
         <v>0</v>
       </c>
       <c r="F45" s="4" t="inlineStr"/>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H45" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="5" t="inlineStr">
@@ -8529,6 +9180,21 @@
           <t>Required columns present.</t>
         </is>
       </c>
+      <c r="G46" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I46" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -8551,6 +9217,21 @@
         <v>0</v>
       </c>
       <c r="F47" s="4" t="inlineStr"/>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H47" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I47" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
@@ -8573,6 +9254,21 @@
         <v>0</v>
       </c>
       <c r="F48" s="5" t="inlineStr"/>
+      <c r="G48" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H48" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -8595,6 +9291,21 @@
         <v>0</v>
       </c>
       <c r="F49" s="4" t="inlineStr"/>
+      <c r="G49" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H49" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
@@ -8617,6 +9328,21 @@
         <v>0</v>
       </c>
       <c r="F50" s="5" t="inlineStr"/>
+      <c r="G50" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H50" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -8639,6 +9365,21 @@
         <v>0</v>
       </c>
       <c r="F51" s="4" t="inlineStr"/>
+      <c r="G51" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H51" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
@@ -8661,6 +9402,21 @@
         <v>0</v>
       </c>
       <c r="F52" s="5" t="inlineStr"/>
+      <c r="G52" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H52" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I52" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -8683,6 +9439,21 @@
         <v>0</v>
       </c>
       <c r="F53" s="4" t="inlineStr"/>
+      <c r="G53" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H53" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I53" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
@@ -8705,6 +9476,21 @@
         <v>0</v>
       </c>
       <c r="F54" s="5" t="inlineStr"/>
+      <c r="G54" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I54" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -8731,6 +9517,21 @@
           <t>Total losses require a separately declared liquidation policy; never filled or dropped.</t>
         </is>
       </c>
+      <c r="G55" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H55" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I55" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
@@ -8753,6 +9554,21 @@
         <v>0</v>
       </c>
       <c r="F56" s="5" t="inlineStr"/>
+      <c r="G56" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H56" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I56" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -8775,6 +9591,21 @@
         <v>0</v>
       </c>
       <c r="F57" s="4" t="inlineStr"/>
+      <c r="G57" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H57" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I57" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
@@ -8797,6 +9628,21 @@
         <v>0</v>
       </c>
       <c r="F58" s="5" t="inlineStr"/>
+      <c r="G58" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H58" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -8819,6 +9665,21 @@
         <v>0</v>
       </c>
       <c r="F59" s="4" t="inlineStr"/>
+      <c r="G59" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H59" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I59" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
@@ -8841,6 +9702,21 @@
         <v>0</v>
       </c>
       <c r="F60" s="5" t="inlineStr"/>
+      <c r="G60" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H60" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I60" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -8863,6 +9739,21 @@
         <v>0</v>
       </c>
       <c r="F61" s="4" t="inlineStr"/>
+      <c r="G61" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H61" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I61" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
@@ -8885,6 +9776,21 @@
         <v>0</v>
       </c>
       <c r="F62" s="5" t="inlineStr"/>
+      <c r="G62" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H62" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I62" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -8907,6 +9813,21 @@
         <v>0</v>
       </c>
       <c r="F63" s="4" t="inlineStr"/>
+      <c r="G63" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H63" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I63" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
@@ -8929,6 +9850,21 @@
         <v>0</v>
       </c>
       <c r="F64" s="5" t="inlineStr"/>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -8951,6 +9887,21 @@
         <v>0</v>
       </c>
       <c r="F65" s="4" t="inlineStr"/>
+      <c r="G65" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H65" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I65" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
@@ -8973,6 +9924,21 @@
         <v>0</v>
       </c>
       <c r="F66" s="5" t="inlineStr"/>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H66" s="5" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -8995,6 +9961,21 @@
         <v>0</v>
       </c>
       <c r="F67" s="4" t="inlineStr"/>
+      <c r="G67" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H67" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I67" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
@@ -9017,6 +9998,21 @@
         <v>0</v>
       </c>
       <c r="F68" s="5" t="inlineStr"/>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H68" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I68" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -9039,6 +10035,21 @@
         <v>0</v>
       </c>
       <c r="F69" s="4" t="inlineStr"/>
+      <c r="G69" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
+      <c r="I69" s="4" t="inlineStr">
+        <is>
+          <t>Risk and constraints</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
@@ -9061,6 +10072,21 @@
         <v>0</v>
       </c>
       <c r="F70" s="5" t="inlineStr"/>
+      <c r="G70" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H70" s="5" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
+      <c r="I70" s="5" t="inlineStr">
+        <is>
+          <t>Risk and constraints</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -9083,6 +10109,21 @@
         <v>0</v>
       </c>
       <c r="F71" s="4" t="inlineStr"/>
+      <c r="G71" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H71" s="4" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I71" s="4" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
@@ -9109,6 +10150,21 @@
           <t>Exactly the declared trailing observations, ending strictly before execution.</t>
         </is>
       </c>
+      <c r="G72" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H72" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I72" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -9131,6 +10187,21 @@
         <v>1e-10</v>
       </c>
       <c r="F73" s="4" t="inlineStr"/>
+      <c r="G73" s="4" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
+      <c r="I73" s="4" t="inlineStr">
+        <is>
+          <t>Risk and constraints</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
@@ -9153,6 +10224,21 @@
         <v>2e-06</v>
       </c>
       <c r="F74" s="5" t="inlineStr"/>
+      <c r="G74" s="5" t="inlineStr">
+        <is>
+          <t>weight fraction</t>
+        </is>
+      </c>
+      <c r="H74" s="5" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
+      <c r="I74" s="5" t="inlineStr">
+        <is>
+          <t>Risk and constraints</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
@@ -9175,6 +10261,21 @@
         <v>2e-06</v>
       </c>
       <c r="F75" s="4" t="inlineStr"/>
+      <c r="G75" s="4" t="inlineStr">
+        <is>
+          <t>weight fraction</t>
+        </is>
+      </c>
+      <c r="H75" s="4" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
+      <c r="I75" s="4" t="inlineStr">
+        <is>
+          <t>Risk and constraints</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
@@ -9197,6 +10298,21 @@
         <v>1e-10</v>
       </c>
       <c r="F76" s="5" t="inlineStr"/>
+      <c r="G76" s="5" t="inlineStr">
+        <is>
+          <t>annual TE fraction</t>
+        </is>
+      </c>
+      <c r="H76" s="5" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
+      <c r="I76" s="5" t="inlineStr">
+        <is>
+          <t>Risk and constraints</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
@@ -9219,6 +10335,21 @@
         <v>2e-06</v>
       </c>
       <c r="F77" s="4" t="inlineStr"/>
+      <c r="G77" s="4" t="inlineStr">
+        <is>
+          <t>annual TE fraction</t>
+        </is>
+      </c>
+      <c r="H77" s="4" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
+      <c r="I77" s="4" t="inlineStr">
+        <is>
+          <t>Risk and constraints</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
@@ -9245,6 +10376,21 @@
           <t>Reconciles the saved Minimum risk solution; does not independently certify optimizer optimality.</t>
         </is>
       </c>
+      <c r="G78" s="5" t="inlineStr">
+        <is>
+          <t>annual TE fraction</t>
+        </is>
+      </c>
+      <c r="H78" s="5" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
+      <c r="I78" s="5" t="inlineStr">
+        <is>
+          <t>Risk and constraints</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
@@ -9267,6 +10413,21 @@
         <v>1e-10</v>
       </c>
       <c r="F79" s="4" t="inlineStr"/>
+      <c r="G79" s="4" t="inlineStr">
+        <is>
+          <t>annual TE fraction</t>
+        </is>
+      </c>
+      <c r="H79" s="4" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
+      <c r="I79" s="4" t="inlineStr">
+        <is>
+          <t>Risk and constraints</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
@@ -9289,6 +10450,21 @@
         <v>0</v>
       </c>
       <c r="F80" s="5" t="inlineStr"/>
+      <c r="G80" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H80" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I80" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
@@ -9311,6 +10487,21 @@
         <v>0.0001</v>
       </c>
       <c r="F81" s="4" t="inlineStr"/>
+      <c r="G81" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I81" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
@@ -9333,6 +10524,21 @@
         <v>0.0001</v>
       </c>
       <c r="F82" s="5" t="inlineStr"/>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H82" s="5" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I82" s="5" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
@@ -9355,6 +10561,21 @@
         <v>0.0001</v>
       </c>
       <c r="F83" s="4" t="inlineStr"/>
+      <c r="G83" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H83" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I83" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
@@ -9377,6 +10598,21 @@
         <v>0.0001</v>
       </c>
       <c r="F84" s="5" t="inlineStr"/>
+      <c r="G84" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H84" s="5" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I84" s="5" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
@@ -9399,6 +10635,21 @@
         <v>0.0001</v>
       </c>
       <c r="F85" s="4" t="inlineStr"/>
+      <c r="G85" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H85" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I85" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
@@ -9421,6 +10672,21 @@
         <v>0.0001</v>
       </c>
       <c r="F86" s="5" t="inlineStr"/>
+      <c r="G86" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H86" s="5" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I86" s="5" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -9443,6 +10709,21 @@
         <v>0</v>
       </c>
       <c r="F87" s="4" t="inlineStr"/>
+      <c r="G87" s="4" t="inlineStr">
+        <is>
+          <t>rows</t>
+        </is>
+      </c>
+      <c r="H87" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I87" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
@@ -9465,6 +10746,21 @@
         <v>1e-10</v>
       </c>
       <c r="F88" s="5" t="inlineStr"/>
+      <c r="G88" s="5" t="inlineStr">
+        <is>
+          <t>return fraction</t>
+        </is>
+      </c>
+      <c r="H88" s="5" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
@@ -9487,6 +10783,21 @@
         <v>1e-10</v>
       </c>
       <c r="F89" s="4" t="inlineStr"/>
+      <c r="G89" s="4" t="inlineStr">
+        <is>
+          <t>return fraction</t>
+        </is>
+      </c>
+      <c r="H89" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I89" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="5" t="inlineStr">
@@ -9509,6 +10820,21 @@
         <v>1e-10</v>
       </c>
       <c r="F90" s="5" t="inlineStr"/>
+      <c r="G90" s="5" t="inlineStr">
+        <is>
+          <t>return fraction</t>
+        </is>
+      </c>
+      <c r="H90" s="5" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I90" s="5" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
@@ -9531,6 +10857,21 @@
         <v>1e-10</v>
       </c>
       <c r="F91" s="4" t="inlineStr"/>
+      <c r="G91" s="4" t="inlineStr">
+        <is>
+          <t>return fraction</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I91" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="5" t="inlineStr">
@@ -9553,6 +10894,21 @@
         <v>1e-10</v>
       </c>
       <c r="F92" s="5" t="inlineStr"/>
+      <c r="G92" s="5" t="inlineStr">
+        <is>
+          <t>return fraction</t>
+        </is>
+      </c>
+      <c r="H92" s="5" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I92" s="5" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -9575,6 +10931,21 @@
         <v>0</v>
       </c>
       <c r="F93" s="4" t="inlineStr"/>
+      <c r="G93" s="4" t="inlineStr">
+        <is>
+          <t>rows</t>
+        </is>
+      </c>
+      <c r="H93" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I93" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
@@ -9597,6 +10968,21 @@
         <v>0.0001</v>
       </c>
       <c r="F94" s="5" t="inlineStr"/>
+      <c r="G94" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H94" s="5" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I94" s="5" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
@@ -9619,6 +11005,21 @@
         <v>1e-10</v>
       </c>
       <c r="F95" s="4" t="inlineStr"/>
+      <c r="G95" s="4" t="inlineStr">
+        <is>
+          <t>return fraction</t>
+        </is>
+      </c>
+      <c r="H95" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I95" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">
@@ -9641,6 +11042,21 @@
         <v>0</v>
       </c>
       <c r="F96" s="5" t="inlineStr"/>
+      <c r="G96" s="5" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H96" s="5" t="inlineStr">
+        <is>
+          <t>data</t>
+        </is>
+      </c>
+      <c r="I96" s="5" t="inlineStr">
+        <is>
+          <t>Data and chronology</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -9663,6 +11079,21 @@
         <v>0.0001</v>
       </c>
       <c r="F97" s="4" t="inlineStr"/>
+      <c r="G97" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H97" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I97" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="5" t="inlineStr">
@@ -9685,6 +11116,21 @@
         <v>0.0001</v>
       </c>
       <c r="F98" s="5" t="inlineStr"/>
+      <c r="G98" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H98" s="5" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I98" s="5" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
@@ -9707,6 +11153,21 @@
         <v>0.0001</v>
       </c>
       <c r="F99" s="4" t="inlineStr"/>
+      <c r="G99" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H99" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I99" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="5" t="inlineStr">
@@ -9729,6 +11190,21 @@
         <v>0.0001</v>
       </c>
       <c r="F100" s="5" t="inlineStr"/>
+      <c r="G100" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H100" s="5" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I100" s="5" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -9751,6 +11227,21 @@
         <v>2e-06</v>
       </c>
       <c r="F101" s="4" t="inlineStr"/>
+      <c r="G101" s="4" t="inlineStr">
+        <is>
+          <t>weight fraction</t>
+        </is>
+      </c>
+      <c r="H101" s="4" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
+      <c r="I101" s="4" t="inlineStr">
+        <is>
+          <t>Risk and constraints</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
@@ -9773,6 +11264,21 @@
         <v>2e-06</v>
       </c>
       <c r="F102" s="5" t="inlineStr"/>
+      <c r="G102" s="5" t="inlineStr">
+        <is>
+          <t>weight fraction</t>
+        </is>
+      </c>
+      <c r="H102" s="5" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
+      <c r="I102" s="5" t="inlineStr">
+        <is>
+          <t>Risk and constraints</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -9795,6 +11301,21 @@
         <v>0</v>
       </c>
       <c r="F103" s="4" t="inlineStr"/>
+      <c r="G103" s="4" t="inlineStr">
+        <is>
+          <t>flag (0/1)</t>
+        </is>
+      </c>
+      <c r="H103" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I103" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="5" t="inlineStr">
@@ -9817,6 +11338,21 @@
         <v>1e-10</v>
       </c>
       <c r="F104" s="5" t="inlineStr"/>
+      <c r="G104" s="5" t="inlineStr">
+        <is>
+          <t>return fraction</t>
+        </is>
+      </c>
+      <c r="H104" s="5" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I104" s="5" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -9839,6 +11375,21 @@
         <v>1e-10</v>
       </c>
       <c r="F105" s="4" t="inlineStr"/>
+      <c r="G105" s="4" t="inlineStr">
+        <is>
+          <t>return fraction</t>
+        </is>
+      </c>
+      <c r="H105" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I105" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
@@ -9861,6 +11412,21 @@
         <v>1e-10</v>
       </c>
       <c r="F106" s="5" t="inlineStr"/>
+      <c r="G106" s="5" t="inlineStr">
+        <is>
+          <t>return fraction</t>
+        </is>
+      </c>
+      <c r="H106" s="5" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I106" s="5" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
@@ -9883,6 +11449,21 @@
         <v>0.0001</v>
       </c>
       <c r="F107" s="4" t="inlineStr"/>
+      <c r="G107" s="4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H107" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I107" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
@@ -9905,6 +11486,21 @@
         <v>1e-10</v>
       </c>
       <c r="F108" s="5" t="inlineStr"/>
+      <c r="G108" s="5" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="H108" s="5" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I108" s="5" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -9927,6 +11523,21 @@
         <v>1e-10</v>
       </c>
       <c r="F109" s="4" t="inlineStr"/>
+      <c r="G109" s="4" t="inlineStr">
+        <is>
+          <t>fraction</t>
+        </is>
+      </c>
+      <c r="H109" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I109" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
@@ -9949,6 +11560,21 @@
         <v>0.0001</v>
       </c>
       <c r="F110" s="5" t="inlineStr"/>
+      <c r="G110" s="5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H110" s="5" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I110" s="5" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
@@ -9971,6 +11597,21 @@
         <v>1e-10</v>
       </c>
       <c r="F111" s="4" t="inlineStr"/>
+      <c r="G111" s="4" t="inlineStr">
+        <is>
+          <t>return fraction</t>
+        </is>
+      </c>
+      <c r="H111" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I111" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
@@ -9993,6 +11634,21 @@
         <v>1e-10</v>
       </c>
       <c r="F112" s="5" t="inlineStr"/>
+      <c r="G112" s="5" t="inlineStr">
+        <is>
+          <t>return fraction</t>
+        </is>
+      </c>
+      <c r="H112" s="5" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I112" s="5" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
@@ -10015,6 +11671,21 @@
         <v>1e-10</v>
       </c>
       <c r="F113" s="4" t="inlineStr"/>
+      <c r="G113" s="4" t="inlineStr">
+        <is>
+          <t>return fraction</t>
+        </is>
+      </c>
+      <c r="H113" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I113" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="5" t="inlineStr">
@@ -10037,6 +11708,21 @@
         <v>1e-10</v>
       </c>
       <c r="F114" s="5" t="inlineStr"/>
+      <c r="G114" s="5" t="inlineStr">
+        <is>
+          <t>return fraction</t>
+        </is>
+      </c>
+      <c r="H114" s="5" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I114" s="5" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
@@ -10059,6 +11745,21 @@
         <v>1e-10</v>
       </c>
       <c r="F115" s="4" t="inlineStr"/>
+      <c r="G115" s="4" t="inlineStr">
+        <is>
+          <t>return fraction</t>
+        </is>
+      </c>
+      <c r="H115" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I115" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="5" t="inlineStr">
@@ -10081,6 +11782,21 @@
         <v>2e-06</v>
       </c>
       <c r="F116" s="5" t="inlineStr"/>
+      <c r="G116" s="5" t="inlineStr">
+        <is>
+          <t>weight fraction</t>
+        </is>
+      </c>
+      <c r="H116" s="5" t="inlineStr">
+        <is>
+          <t>risk</t>
+        </is>
+      </c>
+      <c r="I116" s="5" t="inlineStr">
+        <is>
+          <t>Risk and constraints</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
@@ -10103,6 +11819,21 @@
         <v>1e-10</v>
       </c>
       <c r="F117" s="4" t="inlineStr"/>
+      <c r="G117" s="4" t="inlineStr">
+        <is>
+          <t>return fraction</t>
+        </is>
+      </c>
+      <c r="H117" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I117" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
@@ -10125,6 +11856,21 @@
         <v>1e-10</v>
       </c>
       <c r="F118" s="5" t="inlineStr"/>
+      <c r="G118" s="5" t="inlineStr">
+        <is>
+          <t>return fraction</t>
+        </is>
+      </c>
+      <c r="H118" s="5" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I118" s="5" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
@@ -10147,9 +11893,24 @@
         <v>1e-10</v>
       </c>
       <c r="F119" s="4" t="inlineStr"/>
+      <c r="G119" s="4" t="inlineStr">
+        <is>
+          <t>return fraction</t>
+        </is>
+      </c>
+      <c r="H119" s="4" t="inlineStr">
+        <is>
+          <t>accounting</t>
+        </is>
+      </c>
+      <c r="I119" s="4" t="inlineStr">
+        <is>
+          <t>Reconciliation and accounting</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F119"/>
+  <autoFilter ref="A4:I119"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -10554,7 +12315,7 @@
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="29" customWidth="1" min="4" max="4"/>
     <col width="26" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
@@ -10636,7 +12397,7 @@
         </is>
       </c>
       <c r="C5" s="8" t="n">
-        <v>0.0291880461179388</v>
+        <v>0.0291880461179389</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>14.73633329348556</v>
@@ -10663,7 +12424,7 @@
         </is>
       </c>
       <c r="C6" s="9" t="n">
-        <v>0.0291880461175103</v>
+        <v>0.02918804611751033</v>
       </c>
       <c r="D6" s="9" t="n">
         <v>14.73633329420609</v>
@@ -10729,7 +12490,7 @@
         <v>7.664147569943802</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>2421529.013660693</v>
+        <v>2421529.013660694</v>
       </c>
     </row>
     <row r="9">
@@ -10774,7 +12535,7 @@
         <v>1.638991450996625</v>
       </c>
       <c r="D10" s="9" t="n">
-        <v>7.245279826304221</v>
+        <v>7.245279826304222</v>
       </c>
       <c r="E10" s="9" t="n">
         <v>0.7245279826304222</v>
@@ -10801,7 +12562,7 @@
         <v>0.689654060751515</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>14.84048247125768</v>
+        <v>14.84048247125769</v>
       </c>
       <c r="E11" s="8" t="n">
         <v>1.484048247125769</v>
@@ -10918,7 +12679,7 @@
         <v>8.050148949645951</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>2527573.740927934</v>
+        <v>2527573.740927935</v>
       </c>
     </row>
     <row r="16">
@@ -11026,7 +12787,7 @@
         <v>8.343127276735697</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>2610885.352813465</v>
+        <v>2610885.352813466</v>
       </c>
     </row>
     <row r="20">
@@ -11074,7 +12835,7 @@
         <v>16.97997433376684</v>
       </c>
       <c r="E21" s="8" t="n">
-        <v>1.697997433376684</v>
+        <v>1.697997433376685</v>
       </c>
       <c r="F21" s="8" t="n">
         <v>7.784272196037367</v>
@@ -11215,7 +12976,7 @@
         <v>8.171925591663376</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>2561901.792171228</v>
+        <v>2561901.792171227</v>
       </c>
     </row>
     <row r="27">
@@ -11263,7 +13024,7 @@
         <v>9.792186561612718</v>
       </c>
       <c r="E28" s="9" t="n">
-        <v>0.9792186561612716</v>
+        <v>0.9792186561612717</v>
       </c>
       <c r="F28" s="9" t="n">
         <v>8.394923120198182</v>
@@ -11401,7 +13162,7 @@
         <v>1.696507706803341</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>9.25449796983666</v>
+        <v>9.254497969836661</v>
       </c>
       <c r="G33" s="8" t="n">
         <v>2886401.138245361</v>
@@ -11508,7 +13269,7 @@
         <v>18.23098181024426</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>7.245279826304221</v>
+        <v>7.245279826304222</v>
       </c>
     </row>
     <row r="6">
@@ -14389,17 +16150,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:N34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
     <col width="29" customWidth="1" min="8" max="8"/>
+    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="32" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="29" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -14415,11 +16182,17 @@
       <c r="F1" s="1" t="n"/>
       <c r="G1" s="1" t="n"/>
       <c r="H1" s="1" t="n"/>
+      <c r="I1" s="1" t="n"/>
+      <c r="J1" s="1" t="n"/>
+      <c r="K1" s="1" t="n"/>
+      <c r="L1" s="1" t="n"/>
+      <c r="M1" s="1" t="n"/>
+      <c r="N1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>One aggregate row per account/method, not security-day data. Tracking error is an annual decimal; 0.01 = 1%.</t>
+          <t>One aggregate row per account/method. *_pct fields are percentages; *_bps are basis points. Tracking errors and bound drift are fractions; 0.01 = 1%. NAV/cost totals are USD.</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -14429,6 +16202,12 @@
       <c r="F2" s="2" t="n"/>
       <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
     </row>
     <row r="4" ht="32" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -14453,20 +16232,50 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
+          <t>net_cagr_pct</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>net_volatility_pct</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>max_drawdown_pct</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>annual_one_way_turnover_pct</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>annual_incurred_cost_bps</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
           <t>gross_tracking_error</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>net_tracking_error</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>all_days_weight_limits_drifted</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>interim_drift_days</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>maximum_interim_bound_drift</t>
         </is>
@@ -14490,15 +16299,33 @@
         <v>2579.725145023836</v>
       </c>
       <c r="E5" s="8" t="n">
+        <v>8.074938937491648</v>
+      </c>
+      <c r="F5" s="8" t="n">
+        <v>10.23944339815963</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>-21.91031816316077</v>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>14.73633329348558</v>
+      </c>
+      <c r="I5" s="8" t="n">
+        <v>1.473633329348558</v>
+      </c>
+      <c r="J5" s="8" t="n">
         <v>0.000291880461179384</v>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="K5" s="8" t="n">
         <v>0.0003382763175867321</v>
       </c>
-      <c r="G5" s="4" t="n">
+      <c r="L5" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="8" t="n">
+      <c r="M5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14520,15 +16347,33 @@
         <v>2579.72514518495</v>
       </c>
       <c r="E6" s="9" t="n">
+        <v>8.074938937132758</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>10.23944339775115</v>
+      </c>
+      <c r="G6" s="9" t="n">
+        <v>-21.91031816303591</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>14.73633329420609</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>1.473633329420609</v>
+      </c>
+      <c r="J6" s="9" t="n">
         <v>0.0002918804611750983</v>
       </c>
-      <c r="F6" s="9" t="n">
+      <c r="K6" s="9" t="n">
         <v>0.0003382763174817395</v>
       </c>
-      <c r="G6" s="5" t="n">
+      <c r="L6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="9" t="n">
+      <c r="M6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14550,15 +16395,33 @@
         <v>1418.181434525865</v>
       </c>
       <c r="E7" s="8" t="n">
+        <v>8.278055274888473</v>
+      </c>
+      <c r="F7" s="8" t="n">
+        <v>10.26485847415475</v>
+      </c>
+      <c r="G7" s="8" t="n">
+        <v>-21.87660266991232</v>
+      </c>
+      <c r="H7" s="8" t="n">
+        <v>8.018367322597046</v>
+      </c>
+      <c r="I7" s="8" t="n">
+        <v>0.8018367322597045</v>
+      </c>
+      <c r="J7" s="8" t="n">
         <v>0.002689017476773969</v>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="K7" s="8" t="n">
         <v>0.002690876903665076</v>
       </c>
-      <c r="G7" s="4" t="n">
+      <c r="L7" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H7" s="8" t="n">
+      <c r="M7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14580,15 +16443,33 @@
         <v>2465.788558221965</v>
       </c>
       <c r="E8" s="9" t="n">
+        <v>7.66414756994378</v>
+      </c>
+      <c r="F8" s="9" t="n">
+        <v>11.05346218239021</v>
+      </c>
+      <c r="G8" s="9" t="n">
+        <v>-23.20654059932927</v>
+      </c>
+      <c r="H8" s="9" t="n">
+        <v>14.15410134816056</v>
+      </c>
+      <c r="I8" s="9" t="n">
+        <v>1.415410134816056</v>
+      </c>
+      <c r="J8" s="9" t="n">
         <v>0.01748398542659961</v>
       </c>
-      <c r="F8" s="9" t="n">
+      <c r="K8" s="9" t="n">
         <v>0.0174879344454082</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="L8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H8" s="9" t="n">
+      <c r="M8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14610,15 +16491,33 @@
         <v>3009.621572103092</v>
       </c>
       <c r="E9" s="8" t="n">
+        <v>7.0344434049465</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>10.13208933662559</v>
+      </c>
+      <c r="G9" s="8" t="n">
+        <v>-22.82845883787783</v>
+      </c>
+      <c r="H9" s="8" t="n">
+        <v>18.23098181024423</v>
+      </c>
+      <c r="I9" s="8" t="n">
+        <v>1.823098181024423</v>
+      </c>
+      <c r="J9" s="8" t="n">
         <v>0.01369081354202467</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="K9" s="8" t="n">
         <v>0.0136959883701921</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="L9" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H9" s="8" t="n">
+      <c r="M9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14640,15 +16539,33 @@
         <v>1281.230368381444</v>
       </c>
       <c r="E10" s="9" t="n">
+        <v>7.806281417925365</v>
+      </c>
+      <c r="F10" s="9" t="n">
+        <v>10.34546570093754</v>
+      </c>
+      <c r="G10" s="9" t="n">
+        <v>-23.46368001010863</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>7.245279826304215</v>
+      </c>
+      <c r="I10" s="9" t="n">
+        <v>0.7245279826304216</v>
+      </c>
+      <c r="J10" s="9" t="n">
         <v>0.01638991450996628</v>
       </c>
-      <c r="F10" s="9" t="n">
+      <c r="K10" s="9" t="n">
         <v>0.01639136522151819</v>
       </c>
-      <c r="G10" s="5" t="n">
+      <c r="L10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H10" s="9" t="n">
+      <c r="M10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14670,15 +16587,33 @@
         <v>2615.980667685637</v>
       </c>
       <c r="E11" s="8" t="n">
+        <v>8.211880687061246</v>
+      </c>
+      <c r="F11" s="8" t="n">
+        <v>9.948335432185358</v>
+      </c>
+      <c r="G11" s="8" t="n">
+        <v>-21.38405813444946</v>
+      </c>
+      <c r="H11" s="8" t="n">
+        <v>14.84048247125766</v>
+      </c>
+      <c r="I11" s="8" t="n">
+        <v>1.484048247125766</v>
+      </c>
+      <c r="J11" s="8" t="n">
         <v>0.006896540607515067</v>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="K11" s="8" t="n">
         <v>0.006899257312340247</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="L11" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="M11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14700,15 +16635,33 @@
         <v>2721.725660132361</v>
       </c>
       <c r="E12" s="9" t="n">
+        <v>8.291932072733822</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>10.27598621443682</v>
+      </c>
+      <c r="G12" s="9" t="n">
+        <v>-21.64847728694876</v>
+      </c>
+      <c r="H12" s="9" t="n">
+        <v>15.42444106468334</v>
+      </c>
+      <c r="I12" s="9" t="n">
+        <v>1.542444106468335</v>
+      </c>
+      <c r="J12" s="9" t="n">
         <v>0.005534356093023667</v>
       </c>
-      <c r="F12" s="9" t="n">
+      <c r="K12" s="9" t="n">
         <v>0.005538848615810009</v>
       </c>
-      <c r="G12" s="5" t="n">
+      <c r="L12" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="9" t="n">
+      <c r="M12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14730,15 +16683,33 @@
         <v>1291.17436363583</v>
       </c>
       <c r="E13" s="8" t="n">
+        <v>8.860883173242584</v>
+      </c>
+      <c r="F13" s="8" t="n">
+        <v>10.38379077424082</v>
+      </c>
+      <c r="G13" s="8" t="n">
+        <v>-21.7641075295292</v>
+      </c>
+      <c r="H13" s="8" t="n">
+        <v>6.98526215985455</v>
+      </c>
+      <c r="I13" s="8" t="n">
+        <v>0.6985262159854552</v>
+      </c>
+      <c r="J13" s="8" t="n">
         <v>0.008310308266614781</v>
       </c>
-      <c r="F13" s="8" t="n">
+      <c r="K13" s="8" t="n">
         <v>0.00831057071417959</v>
       </c>
-      <c r="G13" s="4" t="n">
+      <c r="L13" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="8" t="n">
+      <c r="M13" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14760,15 +16731,33 @@
         <v>2540.115715171641</v>
       </c>
       <c r="E14" s="9" t="n">
+        <v>8.37401771217805</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>10.7877776038512</v>
+      </c>
+      <c r="G14" s="9" t="n">
+        <v>-21.42023290327093</v>
+      </c>
+      <c r="H14" s="9" t="n">
+        <v>14.54872785434426</v>
+      </c>
+      <c r="I14" s="9" t="n">
+        <v>1.454872785434427</v>
+      </c>
+      <c r="J14" s="9" t="n">
         <v>0.009477283264071847</v>
       </c>
-      <c r="F14" s="9" t="n">
+      <c r="K14" s="9" t="n">
         <v>0.009480108068439075</v>
       </c>
-      <c r="G14" s="5" t="n">
+      <c r="L14" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="9" t="n">
+      <c r="M14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14790,15 +16779,33 @@
         <v>2735.780778149484</v>
       </c>
       <c r="E15" s="8" t="n">
+        <v>8.050148949645951</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>10.19153767421447</v>
+      </c>
+      <c r="G15" s="8" t="n">
+        <v>-21.30977437040036</v>
+      </c>
+      <c r="H15" s="8" t="n">
+        <v>15.98489535051354</v>
+      </c>
+      <c r="I15" s="8" t="n">
+        <v>1.598489535051354</v>
+      </c>
+      <c r="J15" s="8" t="n">
         <v>0.003102221510946931</v>
       </c>
-      <c r="F15" s="8" t="n">
+      <c r="K15" s="8" t="n">
         <v>0.003110157762711688</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="L15" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="H15" s="8" t="n">
+      <c r="M15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14820,15 +16827,33 @@
         <v>1273.166083686878</v>
       </c>
       <c r="E16" s="9" t="n">
+        <v>8.382774636383239</v>
+      </c>
+      <c r="F16" s="9" t="n">
+        <v>10.13683391528702</v>
+      </c>
+      <c r="G16" s="9" t="n">
+        <v>-21.07614787143568</v>
+      </c>
+      <c r="H16" s="9" t="n">
+        <v>7.30165289647953</v>
+      </c>
+      <c r="I16" s="9" t="n">
+        <v>0.730165289647953</v>
+      </c>
+      <c r="J16" s="9" t="n">
         <v>0.006147348356168236</v>
       </c>
-      <c r="F16" s="9" t="n">
+      <c r="K16" s="9" t="n">
         <v>0.006147780090621768</v>
       </c>
-      <c r="G16" s="5" t="n">
+      <c r="L16" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="H16" s="9" t="n">
+      <c r="M16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="9" t="n">
         <v>0</v>
       </c>
     </row>
@@ -14850,15 +16875,33 @@
         <v>2565.118850661321</v>
       </c>
       <c r="E17" s="8" t="n">
+        <v>7.739946313529611</v>
+      </c>
+      <c r="F17" s="8" t="n">
+        <v>9.701889541091797</v>
+      </c>
+      <c r="G17" s="8" t="n">
+        <v>-21.07874840778634</v>
+      </c>
+      <c r="H17" s="8" t="n">
+        <v>14.96969148667952</v>
+      </c>
+      <c r="I17" s="8" t="n">
+        <v>1.496969148667952</v>
+      </c>
+      <c r="J17" s="8" t="n">
         <v>0.005451189619556276</v>
       </c>
-      <c r="F17" s="8" t="n">
+      <c r="K17" s="8" t="n">
         <v>0.005454124611702307</v>
       </c>
-      <c r="G17" s="4" t="n">
+      <c r="L17" s="4" t="n">
         <v>1754</v>
       </c>
-      <c r="H17" s="8" t="n">
+      <c r="M17" s="4" t="n">
+        <v>1754</v>
+      </c>
+      <c r="N17" s="8" t="n">
         <v>0.01019371113991691</v>
       </c>
     </row>
@@ -14880,15 +16923,33 @@
         <v>2612.136381724718</v>
       </c>
       <c r="E18" s="9" t="n">
+        <v>7.978780304514177</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>10.14385603341743</v>
+      </c>
+      <c r="G18" s="9" t="n">
+        <v>-21.48796546633503</v>
+      </c>
+      <c r="H18" s="9" t="n">
+        <v>15.02722662948243</v>
+      </c>
+      <c r="I18" s="9" t="n">
+        <v>1.502722662948243</v>
+      </c>
+      <c r="J18" s="9" t="n">
         <v>0.001713756094063691</v>
       </c>
-      <c r="F18" s="9" t="n">
+      <c r="K18" s="9" t="n">
         <v>0.001723444262658917</v>
       </c>
-      <c r="G18" s="5" t="n">
+      <c r="L18" s="5" t="n">
         <v>1758</v>
       </c>
-      <c r="H18" s="9" t="n">
+      <c r="M18" s="5" t="n">
+        <v>1758</v>
+      </c>
+      <c r="N18" s="9" t="n">
         <v>0.01058757423842557</v>
       </c>
     </row>
@@ -14910,15 +16971,33 @@
         <v>1281.999203522252</v>
       </c>
       <c r="E19" s="8" t="n">
+        <v>8.343127276735697</v>
+      </c>
+      <c r="F19" s="8" t="n">
+        <v>10.17942463525453</v>
+      </c>
+      <c r="G19" s="8" t="n">
+        <v>-21.5337999584294</v>
+      </c>
+      <c r="H19" s="8" t="n">
+        <v>7.231921636538252</v>
+      </c>
+      <c r="I19" s="8" t="n">
+        <v>0.7231921636538252</v>
+      </c>
+      <c r="J19" s="8" t="n">
         <v>0.004554987872259147</v>
       </c>
-      <c r="F19" s="8" t="n">
+      <c r="K19" s="8" t="n">
         <v>0.004555103262737129</v>
       </c>
-      <c r="G19" s="4" t="n">
+      <c r="L19" s="4" t="n">
         <v>1007</v>
       </c>
-      <c r="H19" s="8" t="n">
+      <c r="M19" s="4" t="n">
+        <v>1007</v>
+      </c>
+      <c r="N19" s="8" t="n">
         <v>0.004017115753815109</v>
       </c>
     </row>
@@ -14940,15 +17019,33 @@
         <v>2512.137128590076</v>
       </c>
       <c r="E20" s="9" t="n">
+        <v>7.064483837520963</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>8.632867745291346</v>
+      </c>
+      <c r="G20" s="9" t="n">
+        <v>-19.40270032919083</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>15.29822186132973</v>
+      </c>
+      <c r="I20" s="9" t="n">
+        <v>1.529822186132972</v>
+      </c>
+      <c r="J20" s="9" t="n">
         <v>0.0162920425345257</v>
       </c>
-      <c r="F20" s="9" t="n">
+      <c r="K20" s="9" t="n">
         <v>0.01629327127299602</v>
       </c>
-      <c r="G20" s="5" t="n">
+      <c r="L20" s="5" t="n">
         <v>1754</v>
       </c>
-      <c r="H20" s="9" t="n">
+      <c r="M20" s="5" t="n">
+        <v>1754</v>
+      </c>
+      <c r="N20" s="9" t="n">
         <v>0.01832976236295328</v>
       </c>
     </row>
@@ -14970,15 +17067,33 @@
         <v>2884.966095369672</v>
       </c>
       <c r="E21" s="8" t="n">
+        <v>7.784272196037412</v>
+      </c>
+      <c r="F21" s="8" t="n">
+        <v>9.95832050282818</v>
+      </c>
+      <c r="G21" s="8" t="n">
+        <v>-20.63901659400865</v>
+      </c>
+      <c r="H21" s="8" t="n">
+        <v>16.97997433376683</v>
+      </c>
+      <c r="I21" s="8" t="n">
+        <v>1.697997433376683</v>
+      </c>
+      <c r="J21" s="8" t="n">
         <v>0.005073109749382462</v>
       </c>
-      <c r="F21" s="8" t="n">
+      <c r="K21" s="8" t="n">
         <v>0.005077731436538761</v>
       </c>
-      <c r="G21" s="4" t="n">
+      <c r="L21" s="4" t="n">
         <v>1759</v>
       </c>
-      <c r="H21" s="8" t="n">
+      <c r="M21" s="4" t="n">
+        <v>1759</v>
+      </c>
+      <c r="N21" s="8" t="n">
         <v>0.02072601704019972</v>
       </c>
     </row>
@@ -15000,15 +17115,33 @@
         <v>1383.540762768428</v>
       </c>
       <c r="E22" s="9" t="n">
+        <v>8.074733043761562</v>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>9.786474158072417</v>
+      </c>
+      <c r="G22" s="9" t="n">
+        <v>-20.26758881878824</v>
+      </c>
+      <c r="H22" s="9" t="n">
+        <v>8.011177441127819</v>
+      </c>
+      <c r="I22" s="9" t="n">
+        <v>0.8011177441127819</v>
+      </c>
+      <c r="J22" s="9" t="n">
         <v>0.008763502823565444</v>
       </c>
-      <c r="F22" s="9" t="n">
+      <c r="K22" s="9" t="n">
         <v>0.00876368150033827</v>
       </c>
-      <c r="G22" s="5" t="n">
+      <c r="L22" s="5" t="n">
         <v>1429</v>
       </c>
-      <c r="H22" s="9" t="n">
+      <c r="M22" s="5" t="n">
+        <v>1429</v>
+      </c>
+      <c r="N22" s="9" t="n">
         <v>0.02038340879725797</v>
       </c>
     </row>
@@ -15030,15 +17163,33 @@
         <v>2494.386491377908</v>
       </c>
       <c r="E23" s="8" t="n">
+        <v>8.868182726311469</v>
+      </c>
+      <c r="F23" s="8" t="n">
+        <v>11.09114821546499</v>
+      </c>
+      <c r="G23" s="8" t="n">
+        <v>-21.97357921685598</v>
+      </c>
+      <c r="H23" s="8" t="n">
+        <v>13.49295241065225</v>
+      </c>
+      <c r="I23" s="8" t="n">
+        <v>1.349295241065225</v>
+      </c>
+      <c r="J23" s="8" t="n">
         <v>0.01235510341820045</v>
       </c>
-      <c r="F23" s="8" t="n">
+      <c r="K23" s="8" t="n">
         <v>0.01235753095433442</v>
       </c>
-      <c r="G23" s="4" t="n">
+      <c r="L23" s="4" t="n">
         <v>1061</v>
       </c>
-      <c r="H23" s="8" t="n">
+      <c r="M23" s="4" t="n">
+        <v>1061</v>
+      </c>
+      <c r="N23" s="8" t="n">
         <v>0.04757793190416892</v>
       </c>
     </row>
@@ -15060,15 +17211,33 @@
         <v>2731.535206999618</v>
       </c>
       <c r="E24" s="9" t="n">
+        <v>8.82507822311438</v>
+      </c>
+      <c r="F24" s="9" t="n">
+        <v>10.39333171696597</v>
+      </c>
+      <c r="G24" s="9" t="n">
+        <v>-21.64533846876157</v>
+      </c>
+      <c r="H24" s="9" t="n">
+        <v>14.74999768482356</v>
+      </c>
+      <c r="I24" s="9" t="n">
+        <v>1.474999768482356</v>
+      </c>
+      <c r="J24" s="9" t="n">
         <v>0.007325890547288934</v>
       </c>
-      <c r="F24" s="9" t="n">
+      <c r="K24" s="9" t="n">
         <v>0.007327831704996808</v>
       </c>
-      <c r="G24" s="5" t="n">
+      <c r="L24" s="5" t="n">
         <v>1080</v>
       </c>
-      <c r="H24" s="9" t="n">
+      <c r="M24" s="5" t="n">
+        <v>1080</v>
+      </c>
+      <c r="N24" s="9" t="n">
         <v>0.05463820796388413</v>
       </c>
     </row>
@@ -15090,15 +17259,33 @@
         <v>1219.839033098505</v>
       </c>
       <c r="E25" s="8" t="n">
+        <v>8.997918890476608</v>
+      </c>
+      <c r="F25" s="8" t="n">
+        <v>10.47041899666461</v>
+      </c>
+      <c r="G25" s="8" t="n">
+        <v>-22.03012601111133</v>
+      </c>
+      <c r="H25" s="8" t="n">
+        <v>6.499750216974312</v>
+      </c>
+      <c r="I25" s="8" t="n">
+        <v>0.6499750216974312</v>
+      </c>
+      <c r="J25" s="8" t="n">
         <v>0.009673029231131135</v>
       </c>
-      <c r="F25" s="8" t="n">
+      <c r="K25" s="8" t="n">
         <v>0.0096727673701935</v>
       </c>
-      <c r="G25" s="4" t="n">
+      <c r="L25" s="4" t="n">
         <v>121</v>
       </c>
-      <c r="H25" s="8" t="n">
+      <c r="M25" s="4" t="n">
+        <v>121</v>
+      </c>
+      <c r="N25" s="8" t="n">
         <v>0.05659163895288705</v>
       </c>
     </row>
@@ -15120,15 +17307,33 @@
         <v>2687.63333478253</v>
       </c>
       <c r="E26" s="9" t="n">
+        <v>8.171925591663353</v>
+      </c>
+      <c r="F26" s="9" t="n">
+        <v>11.28262214772393</v>
+      </c>
+      <c r="G26" s="9" t="n">
+        <v>-22.83797932831957</v>
+      </c>
+      <c r="H26" s="9" t="n">
+        <v>15.22063096617384</v>
+      </c>
+      <c r="I26" s="9" t="n">
+        <v>1.522063096617384</v>
+      </c>
+      <c r="J26" s="9" t="n">
         <v>0.01542254756395396</v>
       </c>
-      <c r="F26" s="9" t="n">
+      <c r="K26" s="9" t="n">
         <v>0.01542511523016283</v>
       </c>
-      <c r="G26" s="5" t="n">
+      <c r="L26" s="5" t="n">
         <v>1369</v>
       </c>
-      <c r="H26" s="9" t="n">
+      <c r="M26" s="5" t="n">
+        <v>1369</v>
+      </c>
+      <c r="N26" s="9" t="n">
         <v>0.03870911186467307</v>
       </c>
     </row>
@@ -15150,15 +17355,33 @@
         <v>3018.730504402243</v>
       </c>
       <c r="E27" s="8" t="n">
+        <v>7.63911464526299</v>
+      </c>
+      <c r="F27" s="8" t="n">
+        <v>10.46838246372237</v>
+      </c>
+      <c r="G27" s="8" t="n">
+        <v>-22.22038401558595</v>
+      </c>
+      <c r="H27" s="8" t="n">
+        <v>17.73598499992384</v>
+      </c>
+      <c r="I27" s="8" t="n">
+        <v>1.773598499992384</v>
+      </c>
+      <c r="J27" s="8" t="n">
         <v>0.0110057919448613</v>
       </c>
-      <c r="F27" s="8" t="n">
+      <c r="K27" s="8" t="n">
         <v>0.01100915548050081</v>
       </c>
-      <c r="G27" s="4" t="n">
+      <c r="L27" s="4" t="n">
         <v>1350</v>
       </c>
-      <c r="H27" s="8" t="n">
+      <c r="M27" s="4" t="n">
+        <v>1350</v>
+      </c>
+      <c r="N27" s="8" t="n">
         <v>0.0414325483934713</v>
       </c>
     </row>
@@ -15180,15 +17403,33 @@
         <v>1792.84234854666</v>
       </c>
       <c r="E28" s="9" t="n">
+        <v>8.394923120198161</v>
+      </c>
+      <c r="F28" s="9" t="n">
+        <v>10.71211305201504</v>
+      </c>
+      <c r="G28" s="9" t="n">
+        <v>-22.65117059158182</v>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>9.792186561612723</v>
+      </c>
+      <c r="I28" s="9" t="n">
+        <v>0.9792186561612721</v>
+      </c>
+      <c r="J28" s="9" t="n">
         <v>0.01360718503265616</v>
       </c>
-      <c r="F28" s="9" t="n">
+      <c r="K28" s="9" t="n">
         <v>0.01360839174822674</v>
       </c>
-      <c r="G28" s="5" t="n">
+      <c r="L28" s="5" t="n">
         <v>1095</v>
       </c>
-      <c r="H28" s="9" t="n">
+      <c r="M28" s="5" t="n">
+        <v>1095</v>
+      </c>
+      <c r="N28" s="9" t="n">
         <v>0.04212962747898383</v>
       </c>
     </row>
@@ -15210,15 +17451,33 @@
         <v>2653.890312534904</v>
       </c>
       <c r="E29" s="8" t="n">
+        <v>7.414596054728229</v>
+      </c>
+      <c r="F29" s="8" t="n">
+        <v>9.766100371722036</v>
+      </c>
+      <c r="G29" s="8" t="n">
+        <v>-22.0847192890109</v>
+      </c>
+      <c r="H29" s="8" t="n">
+        <v>15.98335943519397</v>
+      </c>
+      <c r="I29" s="8" t="n">
+        <v>1.598335943519397</v>
+      </c>
+      <c r="J29" s="8" t="n">
         <v>0.01015167997324464</v>
       </c>
-      <c r="F29" s="8" t="n">
+      <c r="K29" s="8" t="n">
         <v>0.01015177171502499</v>
       </c>
-      <c r="G29" s="4" t="n">
+      <c r="L29" s="4" t="n">
         <v>2535</v>
       </c>
-      <c r="H29" s="8" t="n">
+      <c r="M29" s="4" t="n">
+        <v>2535</v>
+      </c>
+      <c r="N29" s="8" t="n">
         <v>0.04213973834163309</v>
       </c>
     </row>
@@ -15240,15 +17499,33 @@
         <v>2749.360026310408</v>
       </c>
       <c r="E30" s="9" t="n">
+        <v>7.32881743849314</v>
+      </c>
+      <c r="F30" s="9" t="n">
+        <v>10.13513734756653</v>
+      </c>
+      <c r="G30" s="9" t="n">
+        <v>-22.24720743355114</v>
+      </c>
+      <c r="H30" s="9" t="n">
+        <v>16.48783960250465</v>
+      </c>
+      <c r="I30" s="9" t="n">
+        <v>1.648783960250465</v>
+      </c>
+      <c r="J30" s="9" t="n">
         <v>0.007325021777711064</v>
       </c>
-      <c r="F30" s="9" t="n">
+      <c r="K30" s="9" t="n">
         <v>0.007327762642122313</v>
       </c>
-      <c r="G30" s="5" t="n">
+      <c r="L30" s="5" t="n">
         <v>2336</v>
       </c>
-      <c r="H30" s="9" t="n">
+      <c r="M30" s="5" t="n">
+        <v>2336</v>
+      </c>
+      <c r="N30" s="9" t="n">
         <v>0.040852005830701</v>
       </c>
     </row>
@@ -15270,15 +17547,33 @@
         <v>1300.503445573596</v>
       </c>
       <c r="E31" s="8" t="n">
+        <v>7.573212539293883</v>
+      </c>
+      <c r="F31" s="8" t="n">
+        <v>10.1391993945426</v>
+      </c>
+      <c r="G31" s="8" t="n">
+        <v>-22.62377151910955</v>
+      </c>
+      <c r="H31" s="8" t="n">
+        <v>7.880926065371353</v>
+      </c>
+      <c r="I31" s="8" t="n">
+        <v>0.7880926065371353</v>
+      </c>
+      <c r="J31" s="8" t="n">
         <v>0.009916912693656478</v>
       </c>
-      <c r="F31" s="8" t="n">
+      <c r="K31" s="8" t="n">
         <v>0.009917532235428891</v>
       </c>
-      <c r="G31" s="4" t="n">
+      <c r="L31" s="4" t="n">
         <v>1292</v>
       </c>
-      <c r="H31" s="8" t="n">
+      <c r="M31" s="4" t="n">
+        <v>1292</v>
+      </c>
+      <c r="N31" s="8" t="n">
         <v>0.01518494633019682</v>
       </c>
     </row>
@@ -15300,15 +17595,33 @@
         <v>2717.077171568892</v>
       </c>
       <c r="E32" s="9" t="n">
+        <v>7.855735978502798</v>
+      </c>
+      <c r="F32" s="9" t="n">
+        <v>8.313609735955612</v>
+      </c>
+      <c r="G32" s="9" t="n">
+        <v>-18.72508130782467</v>
+      </c>
+      <c r="H32" s="9" t="n">
+        <v>15.55556982440408</v>
+      </c>
+      <c r="I32" s="9" t="n">
+        <v>1.555556982440408</v>
+      </c>
+      <c r="J32" s="9" t="n">
         <v>0.02682463660801744</v>
       </c>
-      <c r="F32" s="9" t="n">
+      <c r="K32" s="9" t="n">
         <v>0.02682513392651383</v>
       </c>
-      <c r="G32" s="5" t="n">
+      <c r="L32" s="5" t="n">
         <v>1790</v>
       </c>
-      <c r="H32" s="9" t="n">
+      <c r="M32" s="5" t="n">
+        <v>1790</v>
+      </c>
+      <c r="N32" s="9" t="n">
         <v>0.01430184990891703</v>
       </c>
     </row>
@@ -15330,15 +17643,33 @@
         <v>3204.214774529888</v>
       </c>
       <c r="E33" s="8" t="n">
+        <v>9.254497969836661</v>
+      </c>
+      <c r="F33" s="8" t="n">
+        <v>10.03997898129288</v>
+      </c>
+      <c r="G33" s="8" t="n">
+        <v>-19.44673938014973</v>
+      </c>
+      <c r="H33" s="8" t="n">
+        <v>16.96507706803343</v>
+      </c>
+      <c r="I33" s="8" t="n">
+        <v>1.696507706803344</v>
+      </c>
+      <c r="J33" s="8" t="n">
         <v>0.01730102880761127</v>
       </c>
-      <c r="F33" s="8" t="n">
+      <c r="K33" s="8" t="n">
         <v>0.01730215184860394</v>
       </c>
-      <c r="G33" s="4" t="n">
+      <c r="L33" s="4" t="n">
         <v>1799</v>
       </c>
-      <c r="H33" s="8" t="n">
+      <c r="M33" s="4" t="n">
+        <v>1799</v>
+      </c>
+      <c r="N33" s="8" t="n">
         <v>0.01703146068817366</v>
       </c>
     </row>
@@ -15360,20 +17691,38 @@
         <v>1160.398700047193</v>
       </c>
       <c r="E34" s="9" t="n">
+        <v>9.155684504757811</v>
+      </c>
+      <c r="F34" s="9" t="n">
+        <v>10.28890859578624</v>
+      </c>
+      <c r="G34" s="9" t="n">
+        <v>-20.11036359163676</v>
+      </c>
+      <c r="H34" s="9" t="n">
+        <v>6.185531783434095</v>
+      </c>
+      <c r="I34" s="9" t="n">
+        <v>0.6185531783434094</v>
+      </c>
+      <c r="J34" s="9" t="n">
         <v>0.01922151858975355</v>
       </c>
-      <c r="F34" s="9" t="n">
+      <c r="K34" s="9" t="n">
         <v>0.01922204994098753</v>
       </c>
-      <c r="G34" s="5" t="n">
+      <c r="L34" s="5" t="n">
         <v>957</v>
       </c>
-      <c r="H34" s="9" t="n">
+      <c r="M34" s="5" t="n">
+        <v>957</v>
+      </c>
+      <c r="N34" s="9" t="n">
         <v>0.005629091773254852</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:H34"/>
+  <autoFilter ref="A4:N34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>

</xml_diff>